<commit_message>
fix: 1.1: File import thêm cột Mã Thiết bị
</commit_message>
<xml_diff>
--- a/src/main/resources/qm/public/resources/measuringEquipmentImportSchema_vi.xlsx
+++ b/src/main/resources/qm/public/resources/measuringEquipmentImportSchema_vi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\qcadoo_demo\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Qcadoo_demo_clone\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A7886EB-CF85-41E5-8BC1-79BCB7BEC890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3AEC2DF-4E75-4067-A29C-07A316217785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4545" yWindow="2715" windowWidth="21600" windowHeight="11235" xr2:uid="{68D7CCB2-5FFD-43FB-9C40-727480D7EABE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68D7CCB2-5FFD-43FB-9C40-727480D7EABE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Thiết bị đo</t>
   </si>
   <si>
     <t>Phương pháp đo</t>
+  </si>
+  <si>
+    <t>Mã thiết bị</t>
   </si>
 </sst>
 </file>
@@ -424,18 +427,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DC442A8-9B14-43DD-AF19-A2F9911D2500}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>